<commit_message>
added 2050 and 55
</commit_message>
<xml_diff>
--- a/inputs/input_data_intertemporal.xlsx
+++ b/inputs/input_data_intertemporal.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Alexander\Studium\EEG\Complementarity Modelling\SolarGeoRisk_EPEC_intertemporal\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B09D3F73-E1D3-47E1-9704-FADEA509A785}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3E25D12-2297-4B62-90BD-0A9C111A788D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4305" yWindow="3975" windowWidth="31530" windowHeight="16905" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="settings" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
     <sheet name="README" sheetId="5" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">params_region!$A$1:$Y$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">params_region!$A$1:$X$7</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -45,7 +45,7 @@
     <author>OpenAI</author>
   </authors>
   <commentList>
-    <comment ref="O1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000001000000}">
+    <comment ref="N1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000001000000}">
       <text>
         <r>
           <rPr>
@@ -59,7 +59,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="P1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000002000000}">
+    <comment ref="O1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000002000000}">
       <text>
         <r>
           <rPr>
@@ -73,7 +73,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Q1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000003000000}">
+    <comment ref="P1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000003000000}">
       <text>
         <r>
           <rPr>
@@ -87,7 +87,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="R1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000004000000}">
+    <comment ref="Q1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000004000000}">
       <text>
         <r>
           <rPr>
@@ -101,7 +101,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="S1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000005000000}">
+    <comment ref="R1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000005000000}">
       <text>
         <r>
           <rPr>
@@ -115,7 +115,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="T1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000006000000}">
+    <comment ref="S1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000006000000}">
       <text>
         <r>
           <rPr>
@@ -129,7 +129,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="U1" authorId="0" shapeId="0" xr:uid="{3BD3B233-C8F3-4C4E-A8E9-4D00AB9FAA5A}">
+    <comment ref="T1" authorId="0" shapeId="0" xr:uid="{3BD3B233-C8F3-4C4E-A8E9-4D00AB9FAA5A}">
       <text>
         <r>
           <rPr>
@@ -143,7 +143,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="V1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000007000000}">
+    <comment ref="U1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000007000000}">
       <text>
         <r>
           <rPr>
@@ -157,7 +157,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="W1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000008000000}">
+    <comment ref="V1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000008000000}">
       <text>
         <r>
           <rPr>
@@ -171,7 +171,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="X1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000009000000}">
+    <comment ref="W1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000009000000}">
       <text>
         <r>
           <rPr>
@@ -185,7 +185,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Y1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-00000A000000}">
+    <comment ref="X1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-00000A000000}">
       <text>
         <r>
           <rPr>
@@ -199,7 +199,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Z1" authorId="0" shapeId="0" xr:uid="{2C5B7B49-3F16-4D84-B7A7-EAEBC7F68F01}">
+    <comment ref="Y1" authorId="0" shapeId="0" xr:uid="{2C5B7B49-3F16-4D84-B7A7-EAEBC7F68F01}">
       <text>
         <r>
           <rPr>
@@ -218,7 +218,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="54">
   <si>
     <t>setting</t>
   </si>
@@ -393,9 +393,6 @@
   </si>
   <si>
     <t>a_dem_2045_usd_per_kw</t>
-  </si>
-  <si>
-    <t>dmax_2045_gw</t>
   </si>
 </sst>
 </file>
@@ -477,7 +474,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -493,6 +490,7 @@
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -520,7 +518,7 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
+      <xdr:col>6</xdr:col>
       <xdr:colOff>1041400</xdr:colOff>
       <xdr:row>33</xdr:row>
       <xdr:rowOff>69850</xdr:rowOff>
@@ -569,7 +567,7 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
+      <xdr:col>6</xdr:col>
       <xdr:colOff>1041400</xdr:colOff>
       <xdr:row>33</xdr:row>
       <xdr:rowOff>69850</xdr:rowOff>
@@ -623,7 +621,7 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
+      <xdr:col>6</xdr:col>
       <xdr:colOff>1041400</xdr:colOff>
       <xdr:row>33</xdr:row>
       <xdr:rowOff>69850</xdr:rowOff>
@@ -677,7 +675,7 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
+      <xdr:col>6</xdr:col>
       <xdr:colOff>1041400</xdr:colOff>
       <xdr:row>33</xdr:row>
       <xdr:rowOff>69850</xdr:rowOff>
@@ -731,7 +729,7 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
+      <xdr:col>6</xdr:col>
       <xdr:colOff>1041400</xdr:colOff>
       <xdr:row>33</xdr:row>
       <xdr:rowOff>69850</xdr:rowOff>
@@ -785,7 +783,7 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
+      <xdr:col>6</xdr:col>
       <xdr:colOff>1041400</xdr:colOff>
       <xdr:row>33</xdr:row>
       <xdr:rowOff>69850</xdr:rowOff>
@@ -839,7 +837,7 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
+      <xdr:col>6</xdr:col>
       <xdr:colOff>1041400</xdr:colOff>
       <xdr:row>33</xdr:row>
       <xdr:rowOff>69850</xdr:rowOff>
@@ -893,7 +891,7 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
+      <xdr:col>6</xdr:col>
       <xdr:colOff>1041400</xdr:colOff>
       <xdr:row>33</xdr:row>
       <xdr:rowOff>69850</xdr:rowOff>
@@ -947,7 +945,7 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
+      <xdr:col>6</xdr:col>
       <xdr:colOff>1041400</xdr:colOff>
       <xdr:row>33</xdr:row>
       <xdr:rowOff>69850</xdr:rowOff>
@@ -1001,7 +999,7 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
+      <xdr:col>6</xdr:col>
       <xdr:colOff>1041400</xdr:colOff>
       <xdr:row>33</xdr:row>
       <xdr:rowOff>69850</xdr:rowOff>
@@ -1055,7 +1053,7 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
+      <xdr:col>6</xdr:col>
       <xdr:colOff>1041400</xdr:colOff>
       <xdr:row>33</xdr:row>
       <xdr:rowOff>69850</xdr:rowOff>
@@ -1109,7 +1107,7 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
+      <xdr:col>6</xdr:col>
       <xdr:colOff>1371600</xdr:colOff>
       <xdr:row>32</xdr:row>
       <xdr:rowOff>66675</xdr:rowOff>
@@ -1131,6 +1129,168 @@
         <a:xfrm>
           <a:off x="0" y="0"/>
           <a:ext cx="8296275" cy="6353175"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>66675</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="13" name="AutoShape 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5EAE2465-B2D2-DB0F-102C-8721179D3A1F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="8277225" cy="6353175"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>66675</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="14" name="AutoShape 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A5F72BF3-E157-8BBA-5332-8560B201DD62}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="8277225" cy="6353175"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>66675</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="15" name="AutoShape 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EE5849E7-9615-192A-5AE6-B395D7A5F35D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="8277225" cy="6353175"/>
         </a:xfrm>
         <a:custGeom>
           <a:avLst/>
@@ -1466,7 +1626,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:Z26"/>
+  <dimension ref="A1:Y26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -1474,29 +1634,28 @@
     <col min="3" max="3" width="21.42578125" customWidth="1"/>
     <col min="4" max="4" width="18.7109375" customWidth="1"/>
     <col min="5" max="6" width="20.28515625" customWidth="1"/>
-    <col min="7" max="7" width="19.42578125" customWidth="1"/>
-    <col min="8" max="8" width="25.7109375" customWidth="1"/>
-    <col min="9" max="9" width="26" customWidth="1"/>
-    <col min="10" max="10" width="30.5703125" customWidth="1"/>
-    <col min="11" max="11" width="20.42578125" customWidth="1"/>
-    <col min="12" max="12" width="23.140625" customWidth="1"/>
-    <col min="13" max="13" width="28" customWidth="1"/>
-    <col min="14" max="14" width="16.5703125" customWidth="1"/>
-    <col min="15" max="15" width="18" customWidth="1"/>
-    <col min="16" max="16" width="27.85546875" customWidth="1"/>
-    <col min="17" max="17" width="25.42578125" customWidth="1"/>
-    <col min="18" max="18" width="24.140625" customWidth="1"/>
-    <col min="19" max="19" width="22.85546875" customWidth="1"/>
-    <col min="20" max="20" width="28.5703125" customWidth="1"/>
-    <col min="21" max="21" width="34.5703125" customWidth="1"/>
-    <col min="22" max="22" width="31.85546875" customWidth="1"/>
-    <col min="23" max="23" width="31.42578125" customWidth="1"/>
-    <col min="24" max="24" width="42.7109375" customWidth="1"/>
-    <col min="25" max="25" width="38.42578125" customWidth="1"/>
-    <col min="26" max="26" width="36.7109375" customWidth="1"/>
+    <col min="7" max="7" width="25.7109375" customWidth="1"/>
+    <col min="8" max="8" width="26" customWidth="1"/>
+    <col min="9" max="9" width="30.5703125" customWidth="1"/>
+    <col min="10" max="10" width="20.42578125" customWidth="1"/>
+    <col min="11" max="11" width="23.140625" customWidth="1"/>
+    <col min="12" max="12" width="28" customWidth="1"/>
+    <col min="13" max="13" width="16.5703125" customWidth="1"/>
+    <col min="14" max="14" width="18" customWidth="1"/>
+    <col min="15" max="15" width="27.85546875" customWidth="1"/>
+    <col min="16" max="16" width="25.42578125" customWidth="1"/>
+    <col min="17" max="17" width="24.140625" customWidth="1"/>
+    <col min="18" max="18" width="22.85546875" customWidth="1"/>
+    <col min="19" max="19" width="28.5703125" customWidth="1"/>
+    <col min="20" max="20" width="34.5703125" customWidth="1"/>
+    <col min="21" max="21" width="31.85546875" customWidth="1"/>
+    <col min="22" max="22" width="31.42578125" customWidth="1"/>
+    <col min="23" max="23" width="42.7109375" customWidth="1"/>
+    <col min="24" max="24" width="38.42578125" customWidth="1"/>
+    <col min="25" max="25" width="36.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>12</v>
       </c>
@@ -1516,67 +1675,64 @@
         <v>30</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>54</v>
+        <v>31</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>32</v>
+        <v>49</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>51</v>
+        <v>33</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="Q1" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="R1" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="S1" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="T1" s="2" t="s">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="U1" s="2" t="s">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="V1" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="W1" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="X1" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Y1" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="Z1" s="2" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -1596,38 +1752,39 @@
         <v>600</v>
       </c>
       <c r="G2">
-        <v>600</v>
+        <v>163</v>
       </c>
       <c r="H2">
-        <v>163</v>
+        <v>50</v>
       </c>
       <c r="I2">
-        <v>50</v>
+        <f>H2*0.05</f>
+        <v>2.5</v>
       </c>
       <c r="J2">
-        <f>I2*0.05</f>
-        <v>2.5</v>
+        <v>27.4</v>
       </c>
       <c r="K2">
-        <v>27.4</v>
+        <v>1</v>
       </c>
       <c r="L2">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="M2">
-        <v>1000</v>
-      </c>
-      <c r="N2">
         <v>1E-3</v>
       </c>
+      <c r="N2" s="5">
+        <v>521.41999999999996</v>
+      </c>
       <c r="O2" s="5">
-        <v>521.41999999999996</v>
+        <v>0.9</v>
       </c>
       <c r="P2" s="5">
-        <v>0.9</v>
+        <f t="shared" ref="P2:T7" si="0">$N2*(1+1/$O2)</f>
+        <v>1100.7755555555555</v>
       </c>
       <c r="Q2" s="5">
-        <f t="shared" ref="Q2:U7" si="0">$O2*(1+1/$P2)</f>
+        <f t="shared" si="0"/>
         <v>1100.7755555555555</v>
       </c>
       <c r="R2" s="5">
@@ -1642,32 +1799,28 @@
         <f t="shared" si="0"/>
         <v>1100.7755555555555</v>
       </c>
-      <c r="U2" s="5">
-        <f t="shared" si="0"/>
-        <v>1100.7755555555555</v>
+      <c r="U2" s="6">
+        <f>$N2/($O2*$C2)</f>
+        <v>2.084012789768185</v>
       </c>
       <c r="V2" s="6">
-        <f>$O2/($P2*$C2)</f>
-        <v>2.084012789768185</v>
+        <f>$N2/($O2*$D2)</f>
+        <v>1.4130623306233061</v>
       </c>
       <c r="W2" s="6">
-        <f>$O2/($P2*$D2)</f>
-        <v>1.4130623306233061</v>
+        <f>$N2/($O2*$E2)</f>
+        <v>1.0728806584362138</v>
       </c>
       <c r="X2" s="6">
-        <f>$O2/($P2*$E2)</f>
-        <v>1.0728806584362138</v>
+        <f>$N2/($O2*$F2)</f>
+        <v>0.96559259259259256</v>
       </c>
       <c r="Y2" s="6">
-        <f>$O2/($P2*$F2)</f>
+        <f>$N2/($O2*$F2)</f>
         <v>0.96559259259259256</v>
       </c>
-      <c r="Z2" s="6">
-        <f>$O2/($P2*$F2)</f>
-        <v>0.96559259259259256</v>
-      </c>
-    </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -1687,35 +1840,36 @@
         <v>250</v>
       </c>
       <c r="G3">
-        <v>250</v>
+        <v>299.25</v>
       </c>
       <c r="H3">
-        <v>299.25</v>
+        <v>175</v>
       </c>
       <c r="I3">
-        <v>175</v>
+        <f t="shared" ref="I3:I7" si="1">H3*0.05</f>
+        <v>8.75</v>
       </c>
       <c r="J3">
-        <f t="shared" ref="J3:J7" si="1">I3*0.05</f>
-        <v>8.75</v>
+        <v>3.6</v>
       </c>
       <c r="K3">
-        <v>3.6</v>
+        <v>1</v>
       </c>
       <c r="L3">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="M3">
-        <v>1000</v>
-      </c>
-      <c r="N3">
         <v>1E-3</v>
       </c>
+      <c r="N3" s="5">
+        <v>967.65</v>
+      </c>
       <c r="O3" s="5">
-        <v>967.65</v>
+        <v>0.9</v>
       </c>
       <c r="P3" s="5">
-        <v>0.9</v>
+        <f t="shared" si="0"/>
+        <v>2042.8166666666666</v>
       </c>
       <c r="Q3" s="5">
         <f t="shared" si="0"/>
@@ -1733,32 +1887,28 @@
         <f t="shared" si="0"/>
         <v>2042.8166666666666</v>
       </c>
-      <c r="U3" s="5">
-        <f t="shared" si="0"/>
-        <v>2042.8166666666666</v>
+      <c r="U3" s="6">
+        <f>$N3/($O3*$C3)</f>
+        <v>18.226253037237949</v>
       </c>
       <c r="V3" s="6">
-        <f>$O3/($P3*$C3)</f>
-        <v>18.226253037237949</v>
+        <f>$N3/($O3*$D3)</f>
+        <v>15.811274509803921</v>
       </c>
       <c r="W3" s="6">
-        <f>$O3/($P3*$D3)</f>
-        <v>15.811274509803921</v>
+        <f>$N3/($O3*$E3)</f>
+        <v>7.4149425287356321</v>
       </c>
       <c r="X3" s="6">
-        <f>$O3/($P3*$E3)</f>
-        <v>7.4149425287356321</v>
+        <f>$N3/($O3*$F3)</f>
+        <v>4.3006666666666664</v>
       </c>
       <c r="Y3" s="6">
-        <f>$O3/($P3*$F3)</f>
+        <f>$N3/($O3*$F3)</f>
         <v>4.3006666666666664</v>
       </c>
-      <c r="Z3" s="6">
-        <f>$O3/($P3*$F3)</f>
-        <v>4.3006666666666664</v>
-      </c>
-    </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -1778,35 +1928,36 @@
         <v>115</v>
       </c>
       <c r="G4">
-        <v>115</v>
+        <v>321.25</v>
       </c>
       <c r="H4">
-        <v>321.25</v>
+        <v>175</v>
       </c>
       <c r="I4">
-        <v>175</v>
-      </c>
-      <c r="J4">
         <f t="shared" si="1"/>
         <v>8.75</v>
       </c>
+      <c r="J4">
+        <v>14.5</v>
+      </c>
       <c r="K4">
-        <v>14.5</v>
+        <v>1</v>
       </c>
       <c r="L4">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="M4">
-        <v>1000</v>
-      </c>
-      <c r="N4">
         <v>1E-3</v>
       </c>
+      <c r="N4" s="5">
+        <v>561.07000000000005</v>
+      </c>
       <c r="O4" s="5">
-        <v>561.07000000000005</v>
+        <v>0.9</v>
       </c>
       <c r="P4" s="5">
-        <v>0.9</v>
+        <f t="shared" si="0"/>
+        <v>1184.4811111111112</v>
       </c>
       <c r="Q4" s="5">
         <f t="shared" si="0"/>
@@ -1824,32 +1975,28 @@
         <f t="shared" si="0"/>
         <v>1184.4811111111112</v>
       </c>
-      <c r="U4" s="5">
-        <f t="shared" si="0"/>
-        <v>1184.4811111111112</v>
+      <c r="U4" s="6">
+        <f>$N4/($O4*$C4)</f>
+        <v>16.289812153412885</v>
       </c>
       <c r="V4" s="6">
-        <f>$O4/($P4*$C4)</f>
-        <v>16.289812153412885</v>
+        <f>$N4/($O4*$D4)</f>
+        <v>8.9058730158730164</v>
       </c>
       <c r="W4" s="6">
-        <f>$O4/($P4*$D4)</f>
-        <v>8.9058730158730164</v>
+        <f>$N4/($O4*$E4)</f>
+        <v>6.5622222222222231</v>
       </c>
       <c r="X4" s="6">
-        <f>$O4/($P4*$E4)</f>
-        <v>6.5622222222222231</v>
+        <f>$N4/($O4*$F4)</f>
+        <v>5.4209661835748797</v>
       </c>
       <c r="Y4" s="6">
-        <f>$O4/($P4*$F4)</f>
+        <f>$N4/($O4*$F4)</f>
         <v>5.4209661835748797</v>
       </c>
-      <c r="Z4" s="6">
-        <f>$O4/($P4*$F4)</f>
-        <v>5.4209661835748797</v>
-      </c>
-    </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>50</v>
       </c>
@@ -1869,35 +2016,36 @@
         <v>460</v>
       </c>
       <c r="G5">
-        <v>460</v>
+        <v>265.75</v>
       </c>
       <c r="H5">
-        <v>265.75204563977178</v>
+        <v>57.5</v>
       </c>
       <c r="I5">
-        <v>57.5</v>
-      </c>
-      <c r="J5">
         <f t="shared" si="1"/>
         <v>2.875</v>
       </c>
+      <c r="J5">
+        <v>3.2479999999999989</v>
+      </c>
       <c r="K5">
-        <v>3.2479999999999989</v>
+        <v>1</v>
       </c>
       <c r="L5">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="M5">
-        <v>1000</v>
-      </c>
-      <c r="N5">
         <v>1E-3</v>
       </c>
+      <c r="N5" s="5">
+        <v>534.14</v>
+      </c>
       <c r="O5" s="5">
-        <v>534.14</v>
+        <v>0.9</v>
       </c>
       <c r="P5" s="5">
-        <v>0.9</v>
+        <f t="shared" si="0"/>
+        <v>1127.6288888888889</v>
       </c>
       <c r="Q5" s="5">
         <f t="shared" si="0"/>
@@ -1915,32 +2063,28 @@
         <f t="shared" si="0"/>
         <v>1127.6288888888889</v>
       </c>
-      <c r="U5" s="5">
-        <f t="shared" si="0"/>
-        <v>1127.6288888888889</v>
+      <c r="U5" s="6">
+        <f>$N5/($O5*$C5)</f>
+        <v>12.092275649732862</v>
       </c>
       <c r="V5" s="6">
-        <f>$O5/($P5*$C5)</f>
-        <v>12.092275649732862</v>
+        <f>$N5/($O5*$D5)</f>
+        <v>2.046513409961686</v>
       </c>
       <c r="W5" s="6">
-        <f>$O5/($P5*$D5)</f>
-        <v>2.046513409961686</v>
+        <f>$N5/($O5*$E5)</f>
+        <v>1.5826370370370371</v>
       </c>
       <c r="X5" s="6">
-        <f>$O5/($P5*$E5)</f>
-        <v>1.5826370370370371</v>
+        <f>$N5/($O5*$F5)</f>
+        <v>1.2901932367149758</v>
       </c>
       <c r="Y5" s="6">
-        <f>$O5/($P5*$F5)</f>
+        <f>$N5/($O5*$F5)</f>
         <v>1.2901932367149758</v>
       </c>
-      <c r="Z5" s="6">
-        <f>$O5/($P5*$F5)</f>
-        <v>1.2901932367149758</v>
-      </c>
-    </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>22</v>
       </c>
@@ -1960,35 +2104,36 @@
         <v>90</v>
       </c>
       <c r="G6">
-        <v>90</v>
+        <v>180.93</v>
       </c>
       <c r="H6">
-        <v>180.93</v>
+        <v>150</v>
       </c>
       <c r="I6">
-        <v>150</v>
-      </c>
-      <c r="J6">
         <f t="shared" si="1"/>
         <v>7.5</v>
       </c>
+      <c r="J6">
+        <v>0.2</v>
+      </c>
       <c r="K6">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="L6">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="M6">
-        <v>1000</v>
-      </c>
-      <c r="N6">
         <v>1E-3</v>
       </c>
+      <c r="N6" s="5">
+        <v>1135.5999999999999</v>
+      </c>
       <c r="O6" s="5">
-        <v>1135.5999999999999</v>
+        <v>0.9</v>
       </c>
       <c r="P6" s="5">
-        <v>0.9</v>
+        <f t="shared" si="0"/>
+        <v>2397.3777777777777</v>
       </c>
       <c r="Q6" s="5">
         <f t="shared" si="0"/>
@@ -2006,32 +2151,28 @@
         <f t="shared" si="0"/>
         <v>2397.3777777777777</v>
       </c>
-      <c r="U6" s="5">
-        <f t="shared" si="0"/>
-        <v>2397.3777777777777</v>
+      <c r="U6" s="6">
+        <f>$N6/($O6*$C6)</f>
+        <v>69.328449328449324</v>
       </c>
       <c r="V6" s="6">
-        <f>$O6/($P6*$C6)</f>
-        <v>69.328449328449324</v>
+        <f>$N6/($O6*$D6)</f>
+        <v>38.235690235690235</v>
       </c>
       <c r="W6" s="6">
-        <f>$O6/($P6*$D6)</f>
-        <v>38.235690235690235</v>
+        <f>$N6/($O6*$E6)</f>
+        <v>20.351254480286734</v>
       </c>
       <c r="X6" s="6">
-        <f>$O6/($P6*$E6)</f>
-        <v>20.351254480286734</v>
+        <f>$N6/($O6*$F6)</f>
+        <v>14.019753086419753</v>
       </c>
       <c r="Y6" s="6">
-        <f>$O6/($P6*$F6)</f>
+        <f>$N6/($O6*$F6)</f>
         <v>14.019753086419753</v>
       </c>
-      <c r="Z6" s="6">
-        <f>$O6/($P6*$F6)</f>
-        <v>14.019753086419753</v>
-      </c>
-    </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>24</v>
       </c>
@@ -2051,35 +2192,36 @@
         <v>180</v>
       </c>
       <c r="G7">
-        <v>180</v>
+        <v>353.38</v>
       </c>
       <c r="H7">
-        <v>353.38</v>
+        <v>125</v>
       </c>
       <c r="I7">
-        <v>125</v>
-      </c>
-      <c r="J7">
         <f t="shared" si="1"/>
         <v>6.25</v>
       </c>
+      <c r="J7">
+        <v>8.6799999999999962</v>
+      </c>
       <c r="K7">
-        <v>8.6799999999999962</v>
+        <v>1</v>
       </c>
       <c r="L7">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="M7">
-        <v>1000</v>
-      </c>
-      <c r="N7">
         <v>1E-3</v>
       </c>
+      <c r="N7" s="5">
+        <v>969.52</v>
+      </c>
       <c r="O7" s="5">
-        <v>969.52</v>
+        <v>0.9</v>
       </c>
       <c r="P7" s="5">
-        <v>0.9</v>
+        <f t="shared" si="0"/>
+        <v>2046.7644444444445</v>
       </c>
       <c r="Q7" s="5">
         <f t="shared" si="0"/>
@@ -2097,77 +2239,75 @@
         <f t="shared" si="0"/>
         <v>2046.7644444444445</v>
       </c>
-      <c r="U7" s="5">
-        <f t="shared" si="0"/>
-        <v>2046.7644444444445</v>
+      <c r="U7" s="6">
+        <f>$N7/($O7*$C7)</f>
+        <v>39.016459414865786</v>
       </c>
       <c r="V7" s="6">
-        <f>$O7/($P7*$C7)</f>
-        <v>39.016459414865786</v>
+        <f>$N7/($O7*$D7)</f>
+        <v>11.895367098547309</v>
       </c>
       <c r="W7" s="6">
-        <f>$O7/($P7*$D7)</f>
-        <v>11.895367098547309</v>
+        <f>$N7/($O7*$E7)</f>
+        <v>8.2864957264957262</v>
       </c>
       <c r="X7" s="6">
-        <f>$O7/($P7*$E7)</f>
-        <v>8.2864957264957262</v>
+        <f>$N7/($O7*$F7)</f>
+        <v>5.9846913580246914</v>
       </c>
       <c r="Y7" s="6">
-        <f>$O7/($P7*$F7)</f>
+        <f>$N7/($O7*$F7)</f>
         <v>5.9846913580246914</v>
       </c>
-      <c r="Z7" s="6">
-        <f>$O7/($P7*$F7)</f>
-        <v>5.9846913580246914</v>
-      </c>
-    </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="T8" s="4"/>
       <c r="U8" s="4"/>
       <c r="V8" s="4"/>
       <c r="W8" s="4"/>
-      <c r="X8" s="4"/>
-    </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="B9" s="7"/>
+    </row>
+    <row r="10" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A10" s="4"/>
       <c r="C10" s="4"/>
     </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A11" s="4"/>
       <c r="C11" s="4"/>
     </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A12" s="4"/>
       <c r="C12" s="4"/>
     </row>
-    <row r="13" spans="1:26" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:25" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="4"/>
       <c r="C13" s="4"/>
     </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A14" s="4"/>
-      <c r="C14" s="4"/>
-    </row>
-    <row r="15" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+    </row>
+    <row r="15" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A15" s="4"/>
-      <c r="C15" s="4"/>
-    </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A16" s="4"/>
-      <c r="C16" s="4"/>
-    </row>
-    <row r="24" spans="19:23" x14ac:dyDescent="0.25">
-      <c r="S24" s="3"/>
-    </row>
-    <row r="25" spans="19:23" x14ac:dyDescent="0.25">
-      <c r="S25" s="3"/>
-    </row>
-    <row r="26" spans="19:23" x14ac:dyDescent="0.25">
+    </row>
+    <row r="24" spans="18:22" x14ac:dyDescent="0.25">
+      <c r="R24" s="3"/>
+    </row>
+    <row r="25" spans="18:22" x14ac:dyDescent="0.25">
+      <c r="R25" s="3"/>
+    </row>
+    <row r="26" spans="18:22" x14ac:dyDescent="0.25">
+      <c r="R26" s="3"/>
       <c r="S26" s="3"/>
       <c r="T26" s="3"/>
       <c r="U26" s="3"/>
       <c r="V26" s="3"/>
-      <c r="W26" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>